<commit_message>
Add PIM module and CI path fixes
</commit_message>
<xml_diff>
--- a/TestData/EmployeeData.xlsx
+++ b/TestData/EmployeeData.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\IC_Projects\Excersise\OrangeHRMHybridAutomationFramework\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D93B9EAC-8B91-482A-9480-8EE9549D25E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7505CDD-49FE-4A98-B97E-C13B90651EF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="EmployeeData" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -70,13 +70,20 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF0A0A0A"/>
+      <name val="Arial Unicode MS"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -99,8 +106,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -383,6 +391,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="4" max="4" width="12.85546875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
@@ -398,7 +409,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>0</v>
       </c>
@@ -408,11 +419,11 @@
       <c r="C2" t="s">
         <v>2</v>
       </c>
-      <c r="D2">
-        <v>123</v>
+      <c r="D2" s="1">
+        <v>102938470</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>3</v>
       </c>
@@ -422,8 +433,8 @@
       <c r="C3" t="s">
         <v>5</v>
       </c>
-      <c r="D3">
-        <v>234</v>
+      <c r="D3" s="1">
+        <v>102938471</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -437,7 +448,7 @@
         <v>8</v>
       </c>
       <c r="D4">
-        <v>567</v>
+        <v>10293842</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
pim code added for screenshots name special characters
</commit_message>
<xml_diff>
--- a/TestData/EmployeeData.xlsx
+++ b/TestData/EmployeeData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\IC_Projects\Excersise\OrangeHRMHybridAutomationFramework\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52CDBC12-3EAF-4092-891F-C583DBF89B3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77BF8FFF-053A-4806-8864-FE74EA4B7F7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -420,7 +420,7 @@
         <v>2</v>
       </c>
       <c r="D2" s="1">
-        <v>10234</v>
+        <v>10230</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
@@ -434,7 +434,7 @@
         <v>5</v>
       </c>
       <c r="D3" s="1">
-        <v>10235</v>
+        <v>10232</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
@@ -448,7 +448,7 @@
         <v>8</v>
       </c>
       <c r="D4">
-        <v>10231</v>
+        <v>1024</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Enhance CI workflow for Node.js 24 and parallel Selenium tests
</commit_message>
<xml_diff>
--- a/TestData/EmployeeData.xlsx
+++ b/TestData/EmployeeData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\IC_Projects\Excersise\OrangeHRMHybridAutomationFramework\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77BF8FFF-053A-4806-8864-FE74EA4B7F7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EBC95C7-1CA4-4B8F-B0A6-D137E043458C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -30,30 +30,6 @@
     <t>John</t>
   </si>
   <si>
-    <t>wick</t>
-  </si>
-  <si>
-    <t>Rex</t>
-  </si>
-  <si>
-    <t>Tony</t>
-  </si>
-  <si>
-    <t>Stark</t>
-  </si>
-  <si>
-    <t>Max</t>
-  </si>
-  <si>
-    <t>Bruce</t>
-  </si>
-  <si>
-    <t>wayne</t>
-  </si>
-  <si>
-    <t>Tob</t>
-  </si>
-  <si>
     <t>FirstName</t>
   </si>
   <si>
@@ -64,6 +40,30 @@
   </si>
   <si>
     <t>EmployeeID</t>
+  </si>
+  <si>
+    <t>Doe</t>
+  </si>
+  <si>
+    <t>Jane</t>
+  </si>
+  <si>
+    <t>Smith</t>
+  </si>
+  <si>
+    <t>Robert</t>
+  </si>
+  <si>
+    <t>Brown</t>
+  </si>
+  <si>
+    <t>A</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>C</t>
   </si>
 </sst>
 </file>
@@ -79,22 +79,27 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
       <color rgb="FF0A0A0A"/>
-      <name val="Arial Unicode MS"/>
+      <name val="Arial"/>
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -102,13 +107,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FFDCDFE5"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -389,67 +411,73 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
+        <v>2</v>
+      </c>
+      <c r="C1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="1">
+        <v>10010</v>
+      </c>
+      <c r="E2" s="2"/>
+    </row>
+    <row r="3" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="1">
+        <v>10011</v>
+      </c>
+      <c r="E3" s="2"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" s="1">
-        <v>10230</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="16.5" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" t="s">
-        <v>4</v>
-      </c>
-      <c r="C3" t="s">
-        <v>5</v>
-      </c>
-      <c r="D3" s="1">
-        <v>10232</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>6</v>
-      </c>
-      <c r="B4" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4">
-        <v>1024</v>
-      </c>
+      <c r="D4" s="3">
+        <v>10012</v>
+      </c>
+      <c r="E4" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Added PIM Employee automation with Excel-driven data, duplicate ID validation, and search verification
</commit_message>
<xml_diff>
--- a/TestData/EmployeeData.xlsx
+++ b/TestData/EmployeeData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\IC_Projects\Excersise\OrangeHRMHybridAutomationFramework\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0EBC95C7-1CA4-4B8F-B0A6-D137E043458C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{18031FB6-EF6F-46B6-A7CB-A05D18192162}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>John</t>
   </si>
@@ -37,9 +37,6 @@
   </si>
   <si>
     <t>LastName</t>
-  </si>
-  <si>
-    <t>EmployeeID</t>
   </si>
   <si>
     <t>Doe</t>
@@ -430,53 +427,44 @@
       <c r="C1" t="s">
         <v>3</v>
       </c>
-      <c r="D1" t="s">
-        <v>4</v>
-      </c>
     </row>
     <row r="2" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D2" s="1">
-        <v>10010</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="D2" s="1"/>
       <c r="E2" s="2"/>
     </row>
     <row r="3" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B3" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="1">
-        <v>10011</v>
-      </c>
+      <c r="D3" s="1"/>
       <c r="E3" s="2"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D4" s="3">
-        <v>10012</v>
-      </c>
+      <c r="D4" s="3"/>
       <c r="E4" s="2"/>
     </row>
   </sheetData>

</xml_diff>